<commit_message>
Reformular justificacion como ampliacion de OC de S/ 27,000 con Estratek
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DoHx9ZQNZXcgog7oJGoyRL
</commit_message>
<xml_diff>
--- a/detalle-gastos-insercion-vehicular.xlsx
+++ b/detalle-gastos-insercion-vehicular.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
-  <si>
-    <t xml:space="preserve">Iniciativa de Insercion Vehicular - Detalle de Gastos para OC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Horizonte: 2.5 meses (75 dias). Escenario que va al documento: 10,000 registros.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+  <si>
+    <t xml:space="preserve">Ampliacion de OC - ESTRATEK S.A.S. SUCURSAL DEL PERU - Iniciativa de Insercion Vehicular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustento del monto de la ampliacion (S/ 27,000 sin IGV) para 75 dias (2.5 meses).</t>
   </si>
   <si>
     <t xml:space="preserve">Leyenda:</t>
@@ -40,13 +40,19 @@
     <t xml:space="preserve">SUPUESTOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Costo plataforma por registro (US$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing digital por registro objetivo (US$) - SUPUESTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bono diario equipo de volanteo (S/) - dato reunion Rodrigo</t>
+    <t xml:space="preserve">Monto de la ampliacion de OC (S/, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros objetivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo plataforma por registro (US$, incluye conversaciones del chatbot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de cambio (S/ por US$) - SUPUESTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bono diario equipo de volanteo (S/)</t>
   </si>
   <si>
     <t xml:space="preserve">Dias que trabaja el equipo por mes</t>
@@ -55,55 +61,40 @@
     <t xml:space="preserve">Meses de ejecucion</t>
   </si>
   <si>
-    <t xml:space="preserve">Tipo de cambio (S/ por US$) - SUPUESTO</t>
-  </si>
-  <si>
     <t xml:space="preserve">IGV</t>
   </si>
   <si>
-    <t xml:space="preserve">DETALLE POR ESCENARIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concepto</t>
+    <t xml:space="preserve">DETALLE DE GASTOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Componente</t>
   </si>
   <si>
     <t xml:space="preserve">Calculo</t>
   </si>
   <si>
-    <t xml:space="preserve">Escenario 5,000 registros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escenario 10,000 registros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registros objetivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta de registros del escenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Plataforma de registros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registros x costo por registro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Marketing digital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registros x presupuesto por registro (amplia la bolsa de recursos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Volanteo (en S/)</t>
+    <t xml:space="preserve">Monto (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Plataforma de registros y chatbot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros x US$ 0.80 x tipo de cambio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Volanteo en campo</t>
   </si>
   <si>
     <t xml:space="preserve">Bono diario x dias/mes x meses</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Volanteo (en US$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monto en S/ / tipo de cambio</t>
+    <t xml:space="preserve">3. Marketing digital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo del monto para campanas de captacion</t>
   </si>
   <si>
     <t xml:space="preserve">VALOR NETO (sin IGV)</t>
@@ -124,34 +115,40 @@
     <t xml:space="preserve">Valor neto + IGV</t>
   </si>
   <si>
-    <t xml:space="preserve">PARTICIPACION DE CADA GASTO (escenario 10,000)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plataforma de registros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing digital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volanteo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo por registro total (US$, sin IGV)</t>
+    <t xml:space="preserve">CONTROLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma en US$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing digital por registro (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo total por registro (S/, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximo de registros que cubre el monto (si marketing = 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validacion</t>
   </si>
   <si>
     <t xml:space="preserve">Notas:</t>
   </si>
   <si>
-    <t xml:space="preserve">- Plataforma: 10,000 registros x US$ 0.80 = US$ 8,000 (dato de la reunion). Si se amplia la meta, solo cambia la fila 'Registros objetivo'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Marketing digital: presupuesto para ampliar la bolsa de recursos y captar registros; aunque parte de los registros llegue por otros canales, se reserva el monto. US$ 0.50/registro es un SUPUESTO: reemplazalo por el monto real.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Volanteo: pago del servicio del equipo de campo (bono de equipo S/150/dia, rango negociado S/120-160) durante 2.5 meses. No depende del numero de registros.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- El monto de la OC es un tope: si no se ejecuta todo, no se gasta. El documento de justificacion usa el escenario de 10,000 registros.</t>
+    <t xml:space="preserve">- ESTRATEK S.A.S. SUCURSAL DEL PERU es el proveedor de la OC: ejecuta la iniciativa de forma integral y coordina a sus aliados especializados. Se emite una sola factura a Calidda.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Plataforma: US$ 0.80 por registro, que incluye las conversaciones del chatbot con el conductor. Se paga solo por registro obtenido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Volanteo: bono de equipo de S/ 150/dia (rango negociado S/ 120-160) durante 2.5 meses. No depende del numero de registros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Marketing digital: es el saldo del monto de la ampliacion. Si cambian los registros o el tipo de cambio, se recalcula solo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- El monto es un tope: si no se llega a los registros objetivo, no se ejecuta todo el gasto.</t>
   </si>
 </sst>
 </file>
@@ -160,13 +157,13 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="&quot;US$ &quot;#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="&quot;S/ &quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="0"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="0%"/>
-    <numFmt numFmtId="171" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;S/ &quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="&quot;US$ &quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0%"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
@@ -290,7 +287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -335,23 +332,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="171" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -363,11 +360,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="172" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -630,9 +635,10 @@
   <dimension ref="A1:D36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -666,39 +672,39 @@
         <v>6</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.8</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>0.5</v>
+      <c r="B7" s="6" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>150</v>
+      <c r="B8" s="7" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>26</v>
+      <c r="B9" s="8" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>2.5</v>
+      <c r="B10" s="5" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -706,7 +712,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="9" t="n">
-        <v>3.4</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -714,250 +720,224 @@
         <v>12</v>
       </c>
       <c r="B12" s="10" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="11" t="n">
         <v>0.18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="12" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="14" t="n">
+        <f aca="false">B7*B8*B9</f>
+        <v>13600</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <f aca="false">C17/$C$20</f>
+        <v>0.503703703703704</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="14" t="n">
-        <f aca="false">C16*$B$6</f>
-        <v>4000</v>
-      </c>
-      <c r="D17" s="14" t="n">
-        <f aca="false">D16*$B$6</f>
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="B18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="C18" s="14" t="n">
+        <f aca="false">B10*B11*B12</f>
+        <v>9750</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <f aca="false">C18/$C$20</f>
+        <v>0.361111111111111</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="14" t="n">
-        <f aca="false">C16*$B$7</f>
-        <v>2500</v>
-      </c>
-      <c r="D18" s="14" t="n">
-        <f aca="false">D16*$B$7</f>
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
+      <c r="B19" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="C19" s="14" t="n">
+        <f aca="false">B6-C17-C18</f>
+        <v>3650</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <f aca="false">C19/$C$20</f>
+        <v>0.135185185185185</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="15" t="n">
-        <f aca="false">$B$8*$B$9*$B$10</f>
-        <v>9750</v>
-      </c>
-      <c r="D19" s="15" t="n">
-        <f aca="false">$B$8*$B$9*$B$10</f>
-        <v>9750</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
+      <c r="B20" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="14" t="n">
-        <f aca="false">C19/$B$11</f>
-        <v>2867.64705882353</v>
-      </c>
-      <c r="D20" s="14" t="n">
-        <f aca="false">D19/$B$11</f>
-        <v>2867.64705882353</v>
+      <c r="C20" s="17" t="n">
+        <f aca="false">C17+C18+C19</f>
+        <v>27000</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">C20/$C$20</f>
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="C21" s="17" t="n">
+        <f aca="false">C20*B13</f>
+        <v>4860</v>
+      </c>
+      <c r="D21" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="17" t="n">
-        <f aca="false">C17+C18+C20</f>
-        <v>9367.64705882353</v>
-      </c>
-      <c r="D21" s="17" t="n">
-        <f aca="false">D17+D18+D20</f>
-        <v>15867.6470588235</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+      <c r="B22" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="C22" s="17" t="n">
+        <f aca="false">C20+C21</f>
+        <v>31860</v>
+      </c>
+      <c r="D22" s="16"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="14" t="n">
-        <f aca="false">C21*$B$12</f>
-        <v>1686.17647058824</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <f aca="false">D21*$B$12</f>
-        <v>2856.17647058824</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="17" t="n">
-        <f aca="false">C21+C22</f>
-        <v>11053.8235294118</v>
-      </c>
-      <c r="D23" s="17" t="n">
-        <f aca="false">D21+D22</f>
-        <v>18723.8235294118</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>34</v>
+      <c r="C25" s="19" t="n">
+        <f aca="false">B7*B8</f>
+        <v>4000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="18" t="n">
-        <f aca="false">D17</f>
-        <v>8000</v>
-      </c>
-      <c r="D26" s="19" t="n">
-        <f aca="false">D17/$D$21</f>
-        <v>0.504170528266914</v>
+        <v>33</v>
+      </c>
+      <c r="C26" s="20" t="n">
+        <f aca="false">C19/B7</f>
+        <v>0.73</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="C27" s="18" t="n">
-        <f aca="false">D18</f>
-        <v>5000</v>
-      </c>
-      <c r="D27" s="19" t="n">
-        <f aca="false">D18/$D$21</f>
-        <v>0.315106580166821</v>
+        <v>34</v>
+      </c>
+      <c r="C27" s="20" t="n">
+        <f aca="false">C20/B7</f>
+        <v>5.4</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <f aca="false">ROUNDDOWN((B6-C18)/(B8*B9),0)</f>
+        <v>6341</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="3" t="str">
+        <f aca="false">IF(C19&lt;0,"El monto no alcanza: baja los registros","OK - el detalle suma el monto de la ampliacion")</f>
+        <v>OK - el detalle suma el monto de la ampliacion</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="18" t="n">
-        <f aca="false">D20</f>
-        <v>2867.64705882353</v>
-      </c>
-      <c r="D28" s="19" t="n">
-        <f aca="false">D20/$D$21</f>
-        <v>0.180722891566265</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="18" t="n">
-        <f aca="false">C21/C16</f>
-        <v>1.87352941176471</v>
-      </c>
-      <c r="D30" s="18" t="n">
-        <f aca="false">D21/D16</f>
-        <v>1.58676470588235</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+    </row>
+    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+    </row>
+    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-    </row>
-    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+    </row>
+    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-    </row>
-    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+    </row>
+    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-    </row>
-    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A35:D35"/>

</xml_diff>